<commit_message>
rm interopsante old thing (#214) 9129a9a78638fddcd0d20eb47eb2f66a9304ba2a
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dp-organization.xlsx
+++ b/main/ig/StructureDefinition-as-dp-organization.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10606" uniqueCount="921">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10606" uniqueCount="920">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-06-07T15:57:22+00:00</t>
+    <t>2024-07-01T19:46:33+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1649,14 +1649,6 @@
   </si>
   <si>
     <t>Organization.identifier:identifiantInterne.type</t>
-  </si>
-  <si>
-    <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
-  &lt;coding&gt;
-    &lt;system value="http://interopsante.org/CodeSystem/fr-v2-0203"/&gt;
-    &lt;code value="INTRN"/&gt;
-  &lt;/coding&gt;
-&lt;/valueCodeableConcept&gt;</t>
   </si>
   <si>
     <t>Organization.identifier:identifiantInterne.system</t>
@@ -17014,7 +17006,7 @@
         <v>78</v>
       </c>
       <c r="S118" t="s" s="2">
-        <v>525</v>
+        <v>500</v>
       </c>
       <c r="T118" t="s" s="2">
         <v>78</v>
@@ -17085,7 +17077,7 @@
     </row>
     <row r="119" hidden="true">
       <c r="A119" t="s" s="2">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B119" t="s" s="2">
         <v>331</v>
@@ -17133,7 +17125,7 @@
         <v>78</v>
       </c>
       <c r="S119" t="s" s="2">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="T119" t="s" s="2">
         <v>336</v>
@@ -17204,7 +17196,7 @@
     </row>
     <row r="120" hidden="true">
       <c r="A120" t="s" s="2">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B120" t="s" s="2">
         <v>341</v>
@@ -17321,7 +17313,7 @@
     </row>
     <row r="121" hidden="true">
       <c r="A121" t="s" s="2">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B121" t="s" s="2">
         <v>350</v>
@@ -17438,7 +17430,7 @@
     </row>
     <row r="122" hidden="true">
       <c r="A122" t="s" s="2">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B122" t="s" s="2">
         <v>359</v>
@@ -17555,10 +17547,10 @@
     </row>
     <row r="123" hidden="true">
       <c r="A123" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -17584,23 +17576,23 @@
         <v>446</v>
       </c>
       <c r="L123" t="s" s="2">
+        <v>531</v>
+      </c>
+      <c r="M123" t="s" s="2">
         <v>532</v>
       </c>
-      <c r="M123" t="s" s="2">
+      <c r="N123" t="s" s="2">
         <v>533</v>
       </c>
-      <c r="N123" t="s" s="2">
+      <c r="O123" t="s" s="2">
         <v>534</v>
       </c>
-      <c r="O123" t="s" s="2">
+      <c r="P123" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q123" t="s" s="2">
         <v>535</v>
       </c>
-      <c r="P123" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q123" t="s" s="2">
-        <v>536</v>
-      </c>
       <c r="R123" t="s" s="2">
         <v>78</v>
       </c>
@@ -17644,7 +17636,7 @@
         <v>78</v>
       </c>
       <c r="AF123" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="AG123" t="s" s="2">
         <v>79</v>
@@ -17662,24 +17654,24 @@
         <v>78</v>
       </c>
       <c r="AL123" t="s" s="2">
+        <v>536</v>
+      </c>
+      <c r="AM123" t="s" s="2">
         <v>537</v>
       </c>
-      <c r="AM123" t="s" s="2">
+      <c r="AN123" t="s" s="2">
         <v>538</v>
       </c>
-      <c r="AN123" t="s" s="2">
+      <c r="AO123" t="s" s="2">
         <v>539</v>
-      </c>
-      <c r="AO123" t="s" s="2">
-        <v>540</v>
       </c>
     </row>
     <row r="124" hidden="true">
       <c r="A124" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -17705,16 +17697,16 @@
         <v>322</v>
       </c>
       <c r="L124" t="s" s="2">
+        <v>541</v>
+      </c>
+      <c r="M124" t="s" s="2">
         <v>542</v>
       </c>
-      <c r="M124" t="s" s="2">
+      <c r="N124" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="N124" t="s" s="2">
+      <c r="O124" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="O124" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="P124" t="s" s="2">
         <v>78</v>
@@ -17742,16 +17734,16 @@
         <v>165</v>
       </c>
       <c r="Y124" t="s" s="2">
+        <v>545</v>
+      </c>
+      <c r="Z124" t="s" s="2">
         <v>546</v>
       </c>
-      <c r="Z124" t="s" s="2">
+      <c r="AA124" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB124" t="s" s="2">
         <v>547</v>
-      </c>
-      <c r="AA124" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB124" t="s" s="2">
-        <v>548</v>
       </c>
       <c r="AC124" s="2"/>
       <c r="AD124" t="s" s="2">
@@ -17761,7 +17753,7 @@
         <v>116</v>
       </c>
       <c r="AF124" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG124" t="s" s="2">
         <v>79</v>
@@ -17779,27 +17771,27 @@
         <v>78</v>
       </c>
       <c r="AL124" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="AM124" t="s" s="2">
         <v>549</v>
-      </c>
-      <c r="AM124" t="s" s="2">
-        <v>550</v>
       </c>
       <c r="AN124" t="s" s="2">
         <v>107</v>
       </c>
       <c r="AO124" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="125" hidden="true">
       <c r="A125" t="s" s="2">
+        <v>551</v>
+      </c>
+      <c r="B125" t="s" s="2">
+        <v>540</v>
+      </c>
+      <c r="C125" t="s" s="2">
         <v>552</v>
-      </c>
-      <c r="B125" t="s" s="2">
-        <v>541</v>
-      </c>
-      <c r="C125" t="s" s="2">
-        <v>553</v>
       </c>
       <c r="D125" t="s" s="2">
         <v>78</v>
@@ -17824,16 +17816,16 @@
         <v>322</v>
       </c>
       <c r="L125" t="s" s="2">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="M125" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="N125" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="N125" t="s" s="2">
+      <c r="O125" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="O125" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="P125" t="s" s="2">
         <v>78</v>
@@ -17862,7 +17854,7 @@
       </c>
       <c r="Y125" s="2"/>
       <c r="Z125" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="AA125" t="s" s="2">
         <v>78</v>
@@ -17880,7 +17872,7 @@
         <v>78</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>79</v>
@@ -17898,24 +17890,24 @@
         <v>78</v>
       </c>
       <c r="AL125" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="AM125" t="s" s="2">
         <v>549</v>
-      </c>
-      <c r="AM125" t="s" s="2">
-        <v>550</v>
       </c>
       <c r="AN125" t="s" s="2">
         <v>107</v>
       </c>
       <c r="AO125" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="126" hidden="true">
       <c r="A126" t="s" s="2">
+        <v>555</v>
+      </c>
+      <c r="B126" t="s" s="2">
         <v>556</v>
-      </c>
-      <c r="B126" t="s" s="2">
-        <v>557</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -18027,10 +18019,10 @@
     </row>
     <row r="127" hidden="true">
       <c r="A127" t="s" s="2">
+        <v>557</v>
+      </c>
+      <c r="B127" t="s" s="2">
         <v>558</v>
-      </c>
-      <c r="B127" t="s" s="2">
-        <v>559</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -18142,13 +18134,13 @@
     </row>
     <row r="128" hidden="true">
       <c r="A128" t="s" s="2">
+        <v>559</v>
+      </c>
+      <c r="B128" t="s" s="2">
+        <v>558</v>
+      </c>
+      <c r="C128" t="s" s="2">
         <v>560</v>
-      </c>
-      <c r="B128" t="s" s="2">
-        <v>559</v>
-      </c>
-      <c r="C128" t="s" s="2">
-        <v>561</v>
       </c>
       <c r="D128" t="s" s="2">
         <v>78</v>
@@ -18170,13 +18162,13 @@
         <v>78</v>
       </c>
       <c r="K128" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="L128" t="s" s="2">
         <v>562</v>
       </c>
-      <c r="L128" t="s" s="2">
+      <c r="M128" t="s" s="2">
         <v>563</v>
-      </c>
-      <c r="M128" t="s" s="2">
-        <v>564</v>
       </c>
       <c r="N128" s="2"/>
       <c r="O128" s="2"/>
@@ -18259,10 +18251,10 @@
     </row>
     <row r="129" hidden="true">
       <c r="A129" t="s" s="2">
+        <v>564</v>
+      </c>
+      <c r="B129" t="s" s="2">
         <v>565</v>
-      </c>
-      <c r="B129" t="s" s="2">
-        <v>566</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" t="s" s="2">
@@ -18374,10 +18366,10 @@
     </row>
     <row r="130" hidden="true">
       <c r="A130" t="s" s="2">
+        <v>566</v>
+      </c>
+      <c r="B130" t="s" s="2">
         <v>567</v>
-      </c>
-      <c r="B130" t="s" s="2">
-        <v>568</v>
       </c>
       <c r="C130" s="2"/>
       <c r="D130" t="s" s="2">
@@ -18489,10 +18481,10 @@
     </row>
     <row r="131" hidden="true">
       <c r="A131" t="s" s="2">
+        <v>568</v>
+      </c>
+      <c r="B131" t="s" s="2">
         <v>569</v>
-      </c>
-      <c r="B131" t="s" s="2">
-        <v>570</v>
       </c>
       <c r="C131" s="2"/>
       <c r="D131" t="s" s="2">
@@ -18532,7 +18524,7 @@
       </c>
       <c r="Q131" s="2"/>
       <c r="R131" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="S131" t="s" s="2">
         <v>78</v>
@@ -18606,10 +18598,10 @@
     </row>
     <row r="132" hidden="true">
       <c r="A132" t="s" s="2">
+        <v>571</v>
+      </c>
+      <c r="B132" t="s" s="2">
         <v>572</v>
-      </c>
-      <c r="B132" t="s" s="2">
-        <v>573</v>
       </c>
       <c r="C132" s="2"/>
       <c r="D132" t="s" s="2">
@@ -18638,7 +18630,7 @@
         <v>231</v>
       </c>
       <c r="M132" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N132" s="2"/>
       <c r="O132" s="2"/>
@@ -18650,7 +18642,7 @@
         <v>78</v>
       </c>
       <c r="S132" t="s" s="2">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="T132" t="s" s="2">
         <v>78</v>
@@ -18669,7 +18661,7 @@
       </c>
       <c r="Y132" s="2"/>
       <c r="Z132" t="s" s="2">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="AA132" t="s" s="2">
         <v>78</v>
@@ -18719,10 +18711,10 @@
     </row>
     <row r="133" hidden="true">
       <c r="A133" t="s" s="2">
+        <v>575</v>
+      </c>
+      <c r="B133" t="s" s="2">
         <v>576</v>
-      </c>
-      <c r="B133" t="s" s="2">
-        <v>577</v>
       </c>
       <c r="C133" s="2"/>
       <c r="D133" t="s" s="2">
@@ -18838,10 +18830,10 @@
     </row>
     <row r="134" hidden="true">
       <c r="A134" t="s" s="2">
+        <v>577</v>
+      </c>
+      <c r="B134" t="s" s="2">
         <v>578</v>
-      </c>
-      <c r="B134" t="s" s="2">
-        <v>579</v>
       </c>
       <c r="C134" s="2"/>
       <c r="D134" t="s" s="2">
@@ -18953,10 +18945,10 @@
     </row>
     <row r="135" hidden="true">
       <c r="A135" t="s" s="2">
+        <v>579</v>
+      </c>
+      <c r="B135" t="s" s="2">
         <v>580</v>
-      </c>
-      <c r="B135" t="s" s="2">
-        <v>581</v>
       </c>
       <c r="C135" s="2"/>
       <c r="D135" t="s" s="2">
@@ -19070,10 +19062,10 @@
     </row>
     <row r="136" hidden="true">
       <c r="A136" t="s" s="2">
+        <v>581</v>
+      </c>
+      <c r="B136" t="s" s="2">
         <v>582</v>
-      </c>
-      <c r="B136" t="s" s="2">
-        <v>583</v>
       </c>
       <c r="C136" s="2"/>
       <c r="D136" t="s" s="2">
@@ -19189,10 +19181,10 @@
     </row>
     <row r="137" hidden="true">
       <c r="A137" t="s" s="2">
+        <v>583</v>
+      </c>
+      <c r="B137" t="s" s="2">
         <v>584</v>
-      </c>
-      <c r="B137" t="s" s="2">
-        <v>585</v>
       </c>
       <c r="C137" s="2"/>
       <c r="D137" t="s" s="2">
@@ -19306,10 +19298,10 @@
     </row>
     <row r="138" hidden="true">
       <c r="A138" t="s" s="2">
+        <v>585</v>
+      </c>
+      <c r="B138" t="s" s="2">
         <v>586</v>
-      </c>
-      <c r="B138" t="s" s="2">
-        <v>587</v>
       </c>
       <c r="C138" s="2"/>
       <c r="D138" t="s" s="2">
@@ -19335,7 +19327,7 @@
         <v>175</v>
       </c>
       <c r="L138" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="M138" t="s" s="2">
         <v>431</v>
@@ -19423,10 +19415,10 @@
     </row>
     <row r="139" hidden="true">
       <c r="A139" t="s" s="2">
+        <v>588</v>
+      </c>
+      <c r="B139" t="s" s="2">
         <v>589</v>
-      </c>
-      <c r="B139" t="s" s="2">
-        <v>590</v>
       </c>
       <c r="C139" s="2"/>
       <c r="D139" t="s" s="2">
@@ -19540,10 +19532,10 @@
     </row>
     <row r="140" hidden="true">
       <c r="A140" t="s" s="2">
+        <v>590</v>
+      </c>
+      <c r="B140" t="s" s="2">
         <v>591</v>
-      </c>
-      <c r="B140" t="s" s="2">
-        <v>592</v>
       </c>
       <c r="C140" s="2"/>
       <c r="D140" t="s" s="2">
@@ -19659,10 +19651,10 @@
     </row>
     <row r="141" hidden="true">
       <c r="A141" t="s" s="2">
+        <v>592</v>
+      </c>
+      <c r="B141" t="s" s="2">
         <v>593</v>
-      </c>
-      <c r="B141" t="s" s="2">
-        <v>594</v>
       </c>
       <c r="C141" s="2"/>
       <c r="D141" t="s" s="2">
@@ -19778,13 +19770,13 @@
     </row>
     <row r="142" hidden="true">
       <c r="A142" t="s" s="2">
+        <v>594</v>
+      </c>
+      <c r="B142" t="s" s="2">
+        <v>540</v>
+      </c>
+      <c r="C142" t="s" s="2">
         <v>595</v>
-      </c>
-      <c r="B142" t="s" s="2">
-        <v>541</v>
-      </c>
-      <c r="C142" t="s" s="2">
-        <v>596</v>
       </c>
       <c r="D142" t="s" s="2">
         <v>78</v>
@@ -19809,16 +19801,16 @@
         <v>322</v>
       </c>
       <c r="L142" t="s" s="2">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="M142" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="N142" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="N142" t="s" s="2">
+      <c r="O142" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="O142" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="P142" t="s" s="2">
         <v>78</v>
@@ -19847,7 +19839,7 @@
       </c>
       <c r="Y142" s="2"/>
       <c r="Z142" t="s" s="2">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="AA142" t="s" s="2">
         <v>78</v>
@@ -19865,7 +19857,7 @@
         <v>78</v>
       </c>
       <c r="AF142" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG142" t="s" s="2">
         <v>79</v>
@@ -19883,24 +19875,24 @@
         <v>78</v>
       </c>
       <c r="AL142" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="AM142" t="s" s="2">
         <v>549</v>
-      </c>
-      <c r="AM142" t="s" s="2">
-        <v>550</v>
       </c>
       <c r="AN142" t="s" s="2">
         <v>107</v>
       </c>
       <c r="AO142" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="143" hidden="true">
       <c r="A143" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B143" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C143" s="2"/>
       <c r="D143" t="s" s="2">
@@ -20012,10 +20004,10 @@
     </row>
     <row r="144" hidden="true">
       <c r="A144" t="s" s="2">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B144" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C144" s="2"/>
       <c r="D144" t="s" s="2">
@@ -20129,10 +20121,10 @@
     </row>
     <row r="145" hidden="true">
       <c r="A145" t="s" s="2">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B145" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C145" s="2"/>
       <c r="D145" t="s" s="2">
@@ -20248,10 +20240,10 @@
     </row>
     <row r="146" hidden="true">
       <c r="A146" t="s" s="2">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B146" t="s" s="2">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C146" s="2"/>
       <c r="D146" t="s" s="2">
@@ -20363,10 +20355,10 @@
     </row>
     <row r="147" hidden="true">
       <c r="A147" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B147" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C147" s="2"/>
       <c r="D147" t="s" s="2">
@@ -20480,10 +20472,10 @@
     </row>
     <row r="148" hidden="true">
       <c r="A148" t="s" s="2">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B148" t="s" s="2">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="C148" s="2"/>
       <c r="D148" t="s" s="2">
@@ -20599,10 +20591,10 @@
     </row>
     <row r="149" hidden="true">
       <c r="A149" t="s" s="2">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B149" t="s" s="2">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C149" s="2"/>
       <c r="D149" t="s" s="2">
@@ -20716,10 +20708,10 @@
     </row>
     <row r="150" hidden="true">
       <c r="A150" t="s" s="2">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B150" t="s" s="2">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C150" s="2"/>
       <c r="D150" t="s" s="2">
@@ -20745,7 +20737,7 @@
         <v>175</v>
       </c>
       <c r="L150" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="M150" t="s" s="2">
         <v>431</v>
@@ -20833,10 +20825,10 @@
     </row>
     <row r="151" hidden="true">
       <c r="A151" t="s" s="2">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B151" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C151" s="2"/>
       <c r="D151" t="s" s="2">
@@ -20950,10 +20942,10 @@
     </row>
     <row r="152" hidden="true">
       <c r="A152" t="s" s="2">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B152" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C152" s="2"/>
       <c r="D152" t="s" s="2">
@@ -21069,10 +21061,10 @@
     </row>
     <row r="153" hidden="true">
       <c r="A153" t="s" s="2">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B153" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C153" s="2"/>
       <c r="D153" t="s" s="2">
@@ -21188,13 +21180,13 @@
     </row>
     <row r="154" hidden="true">
       <c r="A154" t="s" s="2">
+        <v>609</v>
+      </c>
+      <c r="B154" t="s" s="2">
+        <v>540</v>
+      </c>
+      <c r="C154" t="s" s="2">
         <v>610</v>
-      </c>
-      <c r="B154" t="s" s="2">
-        <v>541</v>
-      </c>
-      <c r="C154" t="s" s="2">
-        <v>611</v>
       </c>
       <c r="D154" t="s" s="2">
         <v>78</v>
@@ -21219,16 +21211,16 @@
         <v>322</v>
       </c>
       <c r="L154" t="s" s="2">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="M154" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="N154" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="N154" t="s" s="2">
+      <c r="O154" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="O154" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="P154" t="s" s="2">
         <v>78</v>
@@ -21257,7 +21249,7 @@
       </c>
       <c r="Y154" s="2"/>
       <c r="Z154" t="s" s="2">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AA154" t="s" s="2">
         <v>78</v>
@@ -21275,7 +21267,7 @@
         <v>78</v>
       </c>
       <c r="AF154" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG154" t="s" s="2">
         <v>79</v>
@@ -21293,24 +21285,24 @@
         <v>78</v>
       </c>
       <c r="AL154" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="AM154" t="s" s="2">
         <v>549</v>
-      </c>
-      <c r="AM154" t="s" s="2">
-        <v>550</v>
       </c>
       <c r="AN154" t="s" s="2">
         <v>107</v>
       </c>
       <c r="AO154" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="155" hidden="true">
       <c r="A155" t="s" s="2">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B155" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C155" s="2"/>
       <c r="D155" t="s" s="2">
@@ -21422,10 +21414,10 @@
     </row>
     <row r="156" hidden="true">
       <c r="A156" t="s" s="2">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B156" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C156" s="2"/>
       <c r="D156" t="s" s="2">
@@ -21539,10 +21531,10 @@
     </row>
     <row r="157" hidden="true">
       <c r="A157" t="s" s="2">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B157" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C157" s="2"/>
       <c r="D157" t="s" s="2">
@@ -21658,10 +21650,10 @@
     </row>
     <row r="158" hidden="true">
       <c r="A158" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B158" t="s" s="2">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C158" s="2"/>
       <c r="D158" t="s" s="2">
@@ -21773,10 +21765,10 @@
     </row>
     <row r="159" hidden="true">
       <c r="A159" t="s" s="2">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B159" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C159" s="2"/>
       <c r="D159" t="s" s="2">
@@ -21890,10 +21882,10 @@
     </row>
     <row r="160" hidden="true">
       <c r="A160" t="s" s="2">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B160" t="s" s="2">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="C160" s="2"/>
       <c r="D160" t="s" s="2">
@@ -22009,10 +22001,10 @@
     </row>
     <row r="161" hidden="true">
       <c r="A161" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B161" t="s" s="2">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C161" s="2"/>
       <c r="D161" t="s" s="2">
@@ -22126,10 +22118,10 @@
     </row>
     <row r="162" hidden="true">
       <c r="A162" t="s" s="2">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B162" t="s" s="2">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C162" s="2"/>
       <c r="D162" t="s" s="2">
@@ -22155,7 +22147,7 @@
         <v>175</v>
       </c>
       <c r="L162" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="M162" t="s" s="2">
         <v>431</v>
@@ -22243,10 +22235,10 @@
     </row>
     <row r="163" hidden="true">
       <c r="A163" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B163" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C163" s="2"/>
       <c r="D163" t="s" s="2">
@@ -22360,10 +22352,10 @@
     </row>
     <row r="164" hidden="true">
       <c r="A164" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B164" t="s" s="2">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="C164" s="2"/>
       <c r="D164" t="s" s="2">
@@ -22479,10 +22471,10 @@
     </row>
     <row r="165" hidden="true">
       <c r="A165" t="s" s="2">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B165" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C165" s="2"/>
       <c r="D165" t="s" s="2">
@@ -22598,13 +22590,13 @@
     </row>
     <row r="166" hidden="true">
       <c r="A166" t="s" s="2">
+        <v>624</v>
+      </c>
+      <c r="B166" t="s" s="2">
+        <v>540</v>
+      </c>
+      <c r="C166" t="s" s="2">
         <v>625</v>
-      </c>
-      <c r="B166" t="s" s="2">
-        <v>541</v>
-      </c>
-      <c r="C166" t="s" s="2">
-        <v>626</v>
       </c>
       <c r="D166" t="s" s="2">
         <v>78</v>
@@ -22629,16 +22621,16 @@
         <v>322</v>
       </c>
       <c r="L166" t="s" s="2">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="M166" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="N166" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="N166" t="s" s="2">
+      <c r="O166" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="O166" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="P166" t="s" s="2">
         <v>78</v>
@@ -22667,7 +22659,7 @@
       </c>
       <c r="Y166" s="2"/>
       <c r="Z166" t="s" s="2">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="AA166" t="s" s="2">
         <v>78</v>
@@ -22685,7 +22677,7 @@
         <v>78</v>
       </c>
       <c r="AF166" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG166" t="s" s="2">
         <v>79</v>
@@ -22700,27 +22692,27 @@
         <v>101</v>
       </c>
       <c r="AK166" t="s" s="2">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="AL166" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="AM166" t="s" s="2">
         <v>549</v>
-      </c>
-      <c r="AM166" t="s" s="2">
-        <v>550</v>
       </c>
       <c r="AN166" t="s" s="2">
         <v>107</v>
       </c>
       <c r="AO166" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="167" hidden="true">
       <c r="A167" t="s" s="2">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B167" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C167" s="2"/>
       <c r="D167" t="s" s="2">
@@ -22832,10 +22824,10 @@
     </row>
     <row r="168" hidden="true">
       <c r="A168" t="s" s="2">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B168" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C168" s="2"/>
       <c r="D168" t="s" s="2">
@@ -22947,13 +22939,13 @@
     </row>
     <row r="169" hidden="true">
       <c r="A169" t="s" s="2">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B169" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C169" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D169" t="s" s="2">
         <v>78</v>
@@ -22975,13 +22967,13 @@
         <v>78</v>
       </c>
       <c r="K169" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="L169" t="s" s="2">
         <v>562</v>
       </c>
-      <c r="L169" t="s" s="2">
+      <c r="M169" t="s" s="2">
         <v>563</v>
-      </c>
-      <c r="M169" t="s" s="2">
-        <v>564</v>
       </c>
       <c r="N169" s="2"/>
       <c r="O169" s="2"/>
@@ -23064,10 +23056,10 @@
     </row>
     <row r="170" hidden="true">
       <c r="A170" t="s" s="2">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B170" t="s" s="2">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C170" s="2"/>
       <c r="D170" t="s" s="2">
@@ -23179,10 +23171,10 @@
     </row>
     <row r="171" hidden="true">
       <c r="A171" t="s" s="2">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B171" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C171" s="2"/>
       <c r="D171" t="s" s="2">
@@ -23294,10 +23286,10 @@
     </row>
     <row r="172" hidden="true">
       <c r="A172" t="s" s="2">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B172" t="s" s="2">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C172" s="2"/>
       <c r="D172" t="s" s="2">
@@ -23337,7 +23329,7 @@
       </c>
       <c r="Q172" s="2"/>
       <c r="R172" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="S172" t="s" s="2">
         <v>78</v>
@@ -23411,10 +23403,10 @@
     </row>
     <row r="173" hidden="true">
       <c r="A173" t="s" s="2">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B173" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C173" s="2"/>
       <c r="D173" t="s" s="2">
@@ -23443,7 +23435,7 @@
         <v>231</v>
       </c>
       <c r="M173" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N173" s="2"/>
       <c r="O173" s="2"/>
@@ -23455,7 +23447,7 @@
         <v>78</v>
       </c>
       <c r="S173" t="s" s="2">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="T173" t="s" s="2">
         <v>78</v>
@@ -23474,7 +23466,7 @@
       </c>
       <c r="Y173" s="2"/>
       <c r="Z173" t="s" s="2">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="AA173" t="s" s="2">
         <v>78</v>
@@ -23524,10 +23516,10 @@
     </row>
     <row r="174" hidden="true">
       <c r="A174" t="s" s="2">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B174" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" t="s" s="2">
@@ -23643,10 +23635,10 @@
     </row>
     <row r="175" hidden="true">
       <c r="A175" t="s" s="2">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B175" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C175" s="2"/>
       <c r="D175" t="s" s="2">
@@ -23762,13 +23754,13 @@
     </row>
     <row r="176" hidden="true">
       <c r="A176" t="s" s="2">
+        <v>638</v>
+      </c>
+      <c r="B176" t="s" s="2">
+        <v>540</v>
+      </c>
+      <c r="C176" t="s" s="2">
         <v>639</v>
-      </c>
-      <c r="B176" t="s" s="2">
-        <v>541</v>
-      </c>
-      <c r="C176" t="s" s="2">
-        <v>640</v>
       </c>
       <c r="D176" t="s" s="2">
         <v>78</v>
@@ -23793,16 +23785,16 @@
         <v>322</v>
       </c>
       <c r="L176" t="s" s="2">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="M176" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="N176" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="N176" t="s" s="2">
+      <c r="O176" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="O176" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="P176" t="s" s="2">
         <v>78</v>
@@ -23831,7 +23823,7 @@
       </c>
       <c r="Y176" s="2"/>
       <c r="Z176" t="s" s="2">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="AA176" t="s" s="2">
         <v>78</v>
@@ -23849,7 +23841,7 @@
         <v>78</v>
       </c>
       <c r="AF176" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG176" t="s" s="2">
         <v>79</v>
@@ -23864,27 +23856,27 @@
         <v>101</v>
       </c>
       <c r="AK176" t="s" s="2">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="AL176" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="AM176" t="s" s="2">
         <v>549</v>
-      </c>
-      <c r="AM176" t="s" s="2">
-        <v>550</v>
       </c>
       <c r="AN176" t="s" s="2">
         <v>107</v>
       </c>
       <c r="AO176" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="177" hidden="true">
       <c r="A177" t="s" s="2">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B177" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C177" s="2"/>
       <c r="D177" t="s" s="2">
@@ -23996,10 +23988,10 @@
     </row>
     <row r="178" hidden="true">
       <c r="A178" t="s" s="2">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B178" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" t="s" s="2">
@@ -24111,13 +24103,13 @@
     </row>
     <row r="179" hidden="true">
       <c r="A179" t="s" s="2">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B179" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C179" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D179" t="s" s="2">
         <v>78</v>
@@ -24139,13 +24131,13 @@
         <v>78</v>
       </c>
       <c r="K179" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="L179" t="s" s="2">
         <v>562</v>
       </c>
-      <c r="L179" t="s" s="2">
+      <c r="M179" t="s" s="2">
         <v>563</v>
-      </c>
-      <c r="M179" t="s" s="2">
-        <v>564</v>
       </c>
       <c r="N179" s="2"/>
       <c r="O179" s="2"/>
@@ -24228,10 +24220,10 @@
     </row>
     <row r="180" hidden="true">
       <c r="A180" t="s" s="2">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B180" t="s" s="2">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" t="s" s="2">
@@ -24343,10 +24335,10 @@
     </row>
     <row r="181" hidden="true">
       <c r="A181" t="s" s="2">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="B181" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C181" s="2"/>
       <c r="D181" t="s" s="2">
@@ -24458,10 +24450,10 @@
     </row>
     <row r="182" hidden="true">
       <c r="A182" t="s" s="2">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B182" t="s" s="2">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C182" s="2"/>
       <c r="D182" t="s" s="2">
@@ -24501,7 +24493,7 @@
       </c>
       <c r="Q182" s="2"/>
       <c r="R182" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="S182" t="s" s="2">
         <v>78</v>
@@ -24575,10 +24567,10 @@
     </row>
     <row r="183" hidden="true">
       <c r="A183" t="s" s="2">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B183" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" t="s" s="2">
@@ -24607,7 +24599,7 @@
         <v>231</v>
       </c>
       <c r="M183" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N183" s="2"/>
       <c r="O183" s="2"/>
@@ -24619,7 +24611,7 @@
         <v>78</v>
       </c>
       <c r="S183" t="s" s="2">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="T183" t="s" s="2">
         <v>78</v>
@@ -24638,7 +24630,7 @@
       </c>
       <c r="Y183" s="2"/>
       <c r="Z183" t="s" s="2">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="AA183" t="s" s="2">
         <v>78</v>
@@ -24688,10 +24680,10 @@
     </row>
     <row r="184" hidden="true">
       <c r="A184" t="s" s="2">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B184" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" t="s" s="2">
@@ -24807,10 +24799,10 @@
     </row>
     <row r="185" hidden="true">
       <c r="A185" t="s" s="2">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B185" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" t="s" s="2">
@@ -24926,13 +24918,13 @@
     </row>
     <row r="186" hidden="true">
       <c r="A186" t="s" s="2">
+        <v>652</v>
+      </c>
+      <c r="B186" t="s" s="2">
+        <v>540</v>
+      </c>
+      <c r="C186" t="s" s="2">
         <v>653</v>
-      </c>
-      <c r="B186" t="s" s="2">
-        <v>541</v>
-      </c>
-      <c r="C186" t="s" s="2">
-        <v>654</v>
       </c>
       <c r="D186" t="s" s="2">
         <v>78</v>
@@ -24957,16 +24949,16 @@
         <v>322</v>
       </c>
       <c r="L186" t="s" s="2">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="M186" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="N186" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="N186" t="s" s="2">
+      <c r="O186" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="O186" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="P186" t="s" s="2">
         <v>78</v>
@@ -24995,7 +24987,7 @@
       </c>
       <c r="Y186" s="2"/>
       <c r="Z186" t="s" s="2">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="AA186" t="s" s="2">
         <v>78</v>
@@ -25013,7 +25005,7 @@
         <v>78</v>
       </c>
       <c r="AF186" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG186" t="s" s="2">
         <v>79</v>
@@ -25031,24 +25023,24 @@
         <v>78</v>
       </c>
       <c r="AL186" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="AM186" t="s" s="2">
         <v>549</v>
-      </c>
-      <c r="AM186" t="s" s="2">
-        <v>550</v>
       </c>
       <c r="AN186" t="s" s="2">
         <v>107</v>
       </c>
       <c r="AO186" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="187" hidden="true">
       <c r="A187" t="s" s="2">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B187" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C187" s="2"/>
       <c r="D187" t="s" s="2">
@@ -25160,10 +25152,10 @@
     </row>
     <row r="188" hidden="true">
       <c r="A188" t="s" s="2">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B188" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C188" s="2"/>
       <c r="D188" t="s" s="2">
@@ -25275,13 +25267,13 @@
     </row>
     <row r="189" hidden="true">
       <c r="A189" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B189" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C189" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D189" t="s" s="2">
         <v>78</v>
@@ -25303,13 +25295,13 @@
         <v>78</v>
       </c>
       <c r="K189" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="L189" t="s" s="2">
         <v>562</v>
       </c>
-      <c r="L189" t="s" s="2">
+      <c r="M189" t="s" s="2">
         <v>563</v>
-      </c>
-      <c r="M189" t="s" s="2">
-        <v>564</v>
       </c>
       <c r="N189" s="2"/>
       <c r="O189" s="2"/>
@@ -25392,10 +25384,10 @@
     </row>
     <row r="190" hidden="true">
       <c r="A190" t="s" s="2">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B190" t="s" s="2">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C190" s="2"/>
       <c r="D190" t="s" s="2">
@@ -25507,10 +25499,10 @@
     </row>
     <row r="191" hidden="true">
       <c r="A191" t="s" s="2">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B191" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C191" s="2"/>
       <c r="D191" t="s" s="2">
@@ -25622,10 +25614,10 @@
     </row>
     <row r="192" hidden="true">
       <c r="A192" t="s" s="2">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B192" t="s" s="2">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C192" s="2"/>
       <c r="D192" t="s" s="2">
@@ -25665,7 +25657,7 @@
       </c>
       <c r="Q192" s="2"/>
       <c r="R192" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="S192" t="s" s="2">
         <v>78</v>
@@ -25739,10 +25731,10 @@
     </row>
     <row r="193" hidden="true">
       <c r="A193" t="s" s="2">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B193" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C193" s="2"/>
       <c r="D193" t="s" s="2">
@@ -25771,7 +25763,7 @@
         <v>231</v>
       </c>
       <c r="M193" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N193" s="2"/>
       <c r="O193" s="2"/>
@@ -25783,7 +25775,7 @@
         <v>78</v>
       </c>
       <c r="S193" t="s" s="2">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="T193" t="s" s="2">
         <v>78</v>
@@ -25802,7 +25794,7 @@
       </c>
       <c r="Y193" s="2"/>
       <c r="Z193" t="s" s="2">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="AA193" t="s" s="2">
         <v>78</v>
@@ -25852,10 +25844,10 @@
     </row>
     <row r="194" hidden="true">
       <c r="A194" t="s" s="2">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B194" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C194" s="2"/>
       <c r="D194" t="s" s="2">
@@ -25971,10 +25963,10 @@
     </row>
     <row r="195" hidden="true">
       <c r="A195" t="s" s="2">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B195" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C195" s="2"/>
       <c r="D195" t="s" s="2">
@@ -26090,13 +26082,13 @@
     </row>
     <row r="196" hidden="true">
       <c r="A196" t="s" s="2">
+        <v>665</v>
+      </c>
+      <c r="B196" t="s" s="2">
+        <v>540</v>
+      </c>
+      <c r="C196" t="s" s="2">
         <v>666</v>
-      </c>
-      <c r="B196" t="s" s="2">
-        <v>541</v>
-      </c>
-      <c r="C196" t="s" s="2">
-        <v>667</v>
       </c>
       <c r="D196" t="s" s="2">
         <v>78</v>
@@ -26121,16 +26113,16 @@
         <v>322</v>
       </c>
       <c r="L196" t="s" s="2">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="M196" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="N196" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="N196" t="s" s="2">
+      <c r="O196" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="O196" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="P196" t="s" s="2">
         <v>78</v>
@@ -26158,11 +26150,11 @@
         <v>165</v>
       </c>
       <c r="Y196" t="s" s="2">
+        <v>545</v>
+      </c>
+      <c r="Z196" t="s" s="2">
         <v>546</v>
       </c>
-      <c r="Z196" t="s" s="2">
-        <v>547</v>
-      </c>
       <c r="AA196" t="s" s="2">
         <v>78</v>
       </c>
@@ -26179,7 +26171,7 @@
         <v>78</v>
       </c>
       <c r="AF196" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG196" t="s" s="2">
         <v>79</v>
@@ -26197,24 +26189,24 @@
         <v>78</v>
       </c>
       <c r="AL196" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="AM196" t="s" s="2">
         <v>549</v>
-      </c>
-      <c r="AM196" t="s" s="2">
-        <v>550</v>
       </c>
       <c r="AN196" t="s" s="2">
         <v>107</v>
       </c>
       <c r="AO196" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="197" hidden="true">
       <c r="A197" t="s" s="2">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B197" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C197" s="2"/>
       <c r="D197" t="s" s="2">
@@ -26326,10 +26318,10 @@
     </row>
     <row r="198" hidden="true">
       <c r="A198" t="s" s="2">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B198" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C198" s="2"/>
       <c r="D198" t="s" s="2">
@@ -26441,13 +26433,13 @@
     </row>
     <row r="199" hidden="true">
       <c r="A199" t="s" s="2">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B199" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C199" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D199" t="s" s="2">
         <v>78</v>
@@ -26469,13 +26461,13 @@
         <v>78</v>
       </c>
       <c r="K199" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="L199" t="s" s="2">
         <v>562</v>
       </c>
-      <c r="L199" t="s" s="2">
+      <c r="M199" t="s" s="2">
         <v>563</v>
-      </c>
-      <c r="M199" t="s" s="2">
-        <v>564</v>
       </c>
       <c r="N199" s="2"/>
       <c r="O199" s="2"/>
@@ -26558,10 +26550,10 @@
     </row>
     <row r="200" hidden="true">
       <c r="A200" t="s" s="2">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B200" t="s" s="2">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C200" s="2"/>
       <c r="D200" t="s" s="2">
@@ -26673,10 +26665,10 @@
     </row>
     <row r="201" hidden="true">
       <c r="A201" t="s" s="2">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B201" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C201" s="2"/>
       <c r="D201" t="s" s="2">
@@ -26788,10 +26780,10 @@
     </row>
     <row r="202" hidden="true">
       <c r="A202" t="s" s="2">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="B202" t="s" s="2">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C202" s="2"/>
       <c r="D202" t="s" s="2">
@@ -26831,7 +26823,7 @@
       </c>
       <c r="Q202" s="2"/>
       <c r="R202" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="S202" t="s" s="2">
         <v>78</v>
@@ -26905,10 +26897,10 @@
     </row>
     <row r="203" hidden="true">
       <c r="A203" t="s" s="2">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B203" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C203" s="2"/>
       <c r="D203" t="s" s="2">
@@ -26937,7 +26929,7 @@
         <v>231</v>
       </c>
       <c r="M203" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N203" s="2"/>
       <c r="O203" s="2"/>
@@ -26949,7 +26941,7 @@
         <v>78</v>
       </c>
       <c r="S203" t="s" s="2">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="T203" t="s" s="2">
         <v>78</v>
@@ -26968,7 +26960,7 @@
       </c>
       <c r="Y203" s="2"/>
       <c r="Z203" t="s" s="2">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="AA203" t="s" s="2">
         <v>78</v>
@@ -27018,10 +27010,10 @@
     </row>
     <row r="204" hidden="true">
       <c r="A204" t="s" s="2">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B204" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C204" s="2"/>
       <c r="D204" t="s" s="2">
@@ -27137,10 +27129,10 @@
     </row>
     <row r="205" hidden="true">
       <c r="A205" t="s" s="2">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B205" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C205" s="2"/>
       <c r="D205" t="s" s="2">
@@ -27256,10 +27248,10 @@
     </row>
     <row r="206" hidden="true">
       <c r="A206" t="s" s="2">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B206" t="s" s="2">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="C206" s="2"/>
       <c r="D206" t="s" s="2">
@@ -27285,16 +27277,16 @@
         <v>103</v>
       </c>
       <c r="L206" t="s" s="2">
+        <v>678</v>
+      </c>
+      <c r="M206" t="s" s="2">
         <v>679</v>
       </c>
-      <c r="M206" t="s" s="2">
+      <c r="N206" t="s" s="2">
         <v>680</v>
       </c>
-      <c r="N206" t="s" s="2">
+      <c r="O206" t="s" s="2">
         <v>681</v>
-      </c>
-      <c r="O206" t="s" s="2">
-        <v>682</v>
       </c>
       <c r="P206" t="s" s="2">
         <v>78</v>
@@ -27343,7 +27335,7 @@
         <v>78</v>
       </c>
       <c r="AF206" t="s" s="2">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="AG206" t="s" s="2">
         <v>79</v>
@@ -27358,16 +27350,16 @@
         <v>101</v>
       </c>
       <c r="AK206" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="AL206" t="s" s="2">
         <v>683</v>
       </c>
-      <c r="AL206" t="s" s="2">
+      <c r="AM206" t="s" s="2">
         <v>684</v>
       </c>
-      <c r="AM206" t="s" s="2">
+      <c r="AN206" t="s" s="2">
         <v>685</v>
-      </c>
-      <c r="AN206" t="s" s="2">
-        <v>686</v>
       </c>
       <c r="AO206" t="s" s="2">
         <v>78</v>
@@ -27375,10 +27367,10 @@
     </row>
     <row r="207" hidden="true">
       <c r="A207" t="s" s="2">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B207" t="s" s="2">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="C207" s="2"/>
       <c r="D207" t="s" s="2">
@@ -27404,16 +27396,16 @@
         <v>103</v>
       </c>
       <c r="L207" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="M207" t="s" s="2">
         <v>688</v>
       </c>
-      <c r="M207" t="s" s="2">
+      <c r="N207" t="s" s="2">
         <v>689</v>
       </c>
-      <c r="N207" t="s" s="2">
+      <c r="O207" t="s" s="2">
         <v>690</v>
-      </c>
-      <c r="O207" t="s" s="2">
-        <v>691</v>
       </c>
       <c r="P207" t="s" s="2">
         <v>78</v>
@@ -27462,7 +27454,7 @@
         <v>78</v>
       </c>
       <c r="AF207" t="s" s="2">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="AG207" t="s" s="2">
         <v>79</v>
@@ -27477,13 +27469,13 @@
         <v>101</v>
       </c>
       <c r="AK207" t="s" s="2">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="AL207" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AM207" t="s" s="2">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="AN207" t="s" s="2">
         <v>78</v>
@@ -27494,10 +27486,10 @@
     </row>
     <row r="208" hidden="true">
       <c r="A208" t="s" s="2">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B208" t="s" s="2">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="C208" s="2"/>
       <c r="D208" t="s" s="2">
@@ -27520,19 +27512,19 @@
         <v>78</v>
       </c>
       <c r="K208" t="s" s="2">
+        <v>693</v>
+      </c>
+      <c r="L208" t="s" s="2">
         <v>694</v>
       </c>
-      <c r="L208" t="s" s="2">
+      <c r="M208" t="s" s="2">
         <v>695</v>
       </c>
-      <c r="M208" t="s" s="2">
+      <c r="N208" t="s" s="2">
         <v>696</v>
       </c>
-      <c r="N208" t="s" s="2">
+      <c r="O208" t="s" s="2">
         <v>697</v>
-      </c>
-      <c r="O208" t="s" s="2">
-        <v>698</v>
       </c>
       <c r="P208" t="s" s="2">
         <v>78</v>
@@ -27569,7 +27561,7 @@
         <v>78</v>
       </c>
       <c r="AB208" t="s" s="2">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="AC208" s="2"/>
       <c r="AD208" t="s" s="2">
@@ -27579,7 +27571,7 @@
         <v>116</v>
       </c>
       <c r="AF208" t="s" s="2">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="AG208" t="s" s="2">
         <v>79</v>
@@ -27591,19 +27583,19 @@
         <v>207</v>
       </c>
       <c r="AJ208" t="s" s="2">
+        <v>699</v>
+      </c>
+      <c r="AK208" t="s" s="2">
         <v>700</v>
       </c>
-      <c r="AK208" t="s" s="2">
+      <c r="AL208" t="s" s="2">
         <v>701</v>
       </c>
-      <c r="AL208" t="s" s="2">
+      <c r="AM208" t="s" s="2">
         <v>702</v>
       </c>
-      <c r="AM208" t="s" s="2">
+      <c r="AN208" t="s" s="2">
         <v>703</v>
-      </c>
-      <c r="AN208" t="s" s="2">
-        <v>704</v>
       </c>
       <c r="AO208" t="s" s="2">
         <v>78</v>
@@ -27611,10 +27603,10 @@
     </row>
     <row r="209" hidden="true">
       <c r="A209" t="s" s="2">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="B209" t="s" s="2">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C209" s="2"/>
       <c r="D209" t="s" s="2">
@@ -27726,10 +27718,10 @@
     </row>
     <row r="210" hidden="true">
       <c r="A210" t="s" s="2">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B210" t="s" s="2">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C210" s="2"/>
       <c r="D210" t="s" s="2">
@@ -27843,13 +27835,13 @@
     </row>
     <row r="211" hidden="true">
       <c r="A211" t="s" s="2">
+        <v>706</v>
+      </c>
+      <c r="B211" t="s" s="2">
+        <v>705</v>
+      </c>
+      <c r="C211" t="s" s="2">
         <v>707</v>
-      </c>
-      <c r="B211" t="s" s="2">
-        <v>706</v>
-      </c>
-      <c r="C211" t="s" s="2">
-        <v>708</v>
       </c>
       <c r="D211" t="s" s="2">
         <v>78</v>
@@ -27871,13 +27863,13 @@
         <v>78</v>
       </c>
       <c r="K211" t="s" s="2">
+        <v>708</v>
+      </c>
+      <c r="L211" t="s" s="2">
         <v>709</v>
       </c>
-      <c r="L211" t="s" s="2">
+      <c r="M211" t="s" s="2">
         <v>710</v>
-      </c>
-      <c r="M211" t="s" s="2">
-        <v>711</v>
       </c>
       <c r="N211" s="2"/>
       <c r="O211" s="2"/>
@@ -27960,10 +27952,10 @@
     </row>
     <row r="212" hidden="true">
       <c r="A212" t="s" s="2">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B212" t="s" s="2">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C212" s="2"/>
       <c r="D212" t="s" s="2">
@@ -27989,10 +27981,10 @@
         <v>175</v>
       </c>
       <c r="L212" t="s" s="2">
+        <v>712</v>
+      </c>
+      <c r="M212" t="s" s="2">
         <v>713</v>
-      </c>
-      <c r="M212" t="s" s="2">
-        <v>714</v>
       </c>
       <c r="N212" s="2"/>
       <c r="O212" s="2"/>
@@ -28022,37 +28014,37 @@
         <v>316</v>
       </c>
       <c r="Y212" t="s" s="2">
+        <v>714</v>
+      </c>
+      <c r="Z212" t="s" s="2">
         <v>715</v>
       </c>
-      <c r="Z212" t="s" s="2">
+      <c r="AA212" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB212" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC212" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD212" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE212" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF212" t="s" s="2">
         <v>716</v>
       </c>
-      <c r="AA212" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB212" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC212" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD212" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE212" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF212" t="s" s="2">
+      <c r="AG212" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH212" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI212" t="s" s="2">
         <v>717</v>
-      </c>
-      <c r="AG212" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH212" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI212" t="s" s="2">
-        <v>718</v>
       </c>
       <c r="AJ212" t="s" s="2">
         <v>101</v>
@@ -28061,13 +28053,13 @@
         <v>78</v>
       </c>
       <c r="AL212" t="s" s="2">
+        <v>718</v>
+      </c>
+      <c r="AM212" t="s" s="2">
         <v>719</v>
       </c>
-      <c r="AM212" t="s" s="2">
+      <c r="AN212" t="s" s="2">
         <v>720</v>
-      </c>
-      <c r="AN212" t="s" s="2">
-        <v>721</v>
       </c>
       <c r="AO212" t="s" s="2">
         <v>78</v>
@@ -28075,10 +28067,10 @@
     </row>
     <row r="213" hidden="true">
       <c r="A213" t="s" s="2">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B213" t="s" s="2">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C213" s="2"/>
       <c r="D213" t="s" s="2">
@@ -28104,16 +28096,16 @@
         <v>103</v>
       </c>
       <c r="L213" t="s" s="2">
+        <v>722</v>
+      </c>
+      <c r="M213" t="s" s="2">
         <v>723</v>
       </c>
-      <c r="M213" t="s" s="2">
+      <c r="N213" t="s" s="2">
         <v>724</v>
       </c>
-      <c r="N213" t="s" s="2">
+      <c r="O213" t="s" s="2">
         <v>725</v>
-      </c>
-      <c r="O213" t="s" s="2">
-        <v>726</v>
       </c>
       <c r="P213" t="s" s="2">
         <v>78</v>
@@ -28162,7 +28154,7 @@
         <v>78</v>
       </c>
       <c r="AF213" t="s" s="2">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="AG213" t="s" s="2">
         <v>79</v>
@@ -28180,10 +28172,10 @@
         <v>78</v>
       </c>
       <c r="AL213" t="s" s="2">
+        <v>727</v>
+      </c>
+      <c r="AM213" t="s" s="2">
         <v>728</v>
-      </c>
-      <c r="AM213" t="s" s="2">
-        <v>729</v>
       </c>
       <c r="AN213" t="s" s="2">
         <v>349</v>
@@ -28194,10 +28186,10 @@
     </row>
     <row r="214" hidden="true">
       <c r="A214" t="s" s="2">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B214" t="s" s="2">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="C214" s="2"/>
       <c r="D214" t="s" s="2">
@@ -28223,16 +28215,16 @@
         <v>175</v>
       </c>
       <c r="L214" t="s" s="2">
+        <v>730</v>
+      </c>
+      <c r="M214" t="s" s="2">
         <v>731</v>
       </c>
-      <c r="M214" t="s" s="2">
+      <c r="N214" t="s" s="2">
         <v>732</v>
       </c>
-      <c r="N214" t="s" s="2">
+      <c r="O214" t="s" s="2">
         <v>733</v>
-      </c>
-      <c r="O214" t="s" s="2">
-        <v>734</v>
       </c>
       <c r="P214" t="s" s="2">
         <v>78</v>
@@ -28260,28 +28252,28 @@
         <v>316</v>
       </c>
       <c r="Y214" t="s" s="2">
+        <v>734</v>
+      </c>
+      <c r="Z214" t="s" s="2">
         <v>735</v>
       </c>
-      <c r="Z214" t="s" s="2">
+      <c r="AA214" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB214" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC214" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD214" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE214" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF214" t="s" s="2">
         <v>736</v>
-      </c>
-      <c r="AA214" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB214" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC214" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD214" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE214" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF214" t="s" s="2">
-        <v>737</v>
       </c>
       <c r="AG214" t="s" s="2">
         <v>79</v>
@@ -28299,13 +28291,13 @@
         <v>78</v>
       </c>
       <c r="AL214" t="s" s="2">
+        <v>737</v>
+      </c>
+      <c r="AM214" t="s" s="2">
         <v>738</v>
       </c>
-      <c r="AM214" t="s" s="2">
+      <c r="AN214" t="s" s="2">
         <v>739</v>
-      </c>
-      <c r="AN214" t="s" s="2">
-        <v>740</v>
       </c>
       <c r="AO214" t="s" s="2">
         <v>78</v>
@@ -28313,10 +28305,10 @@
     </row>
     <row r="215" hidden="true">
       <c r="A215" t="s" s="2">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B215" t="s" s="2">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="C215" s="2"/>
       <c r="D215" t="s" s="2">
@@ -28339,16 +28331,16 @@
         <v>90</v>
       </c>
       <c r="K215" t="s" s="2">
+        <v>741</v>
+      </c>
+      <c r="L215" t="s" s="2">
         <v>742</v>
       </c>
-      <c r="L215" t="s" s="2">
+      <c r="M215" t="s" s="2">
         <v>743</v>
       </c>
-      <c r="M215" t="s" s="2">
+      <c r="N215" t="s" s="2">
         <v>744</v>
-      </c>
-      <c r="N215" t="s" s="2">
-        <v>745</v>
       </c>
       <c r="O215" s="2"/>
       <c r="P215" t="s" s="2">
@@ -28398,7 +28390,7 @@
         <v>78</v>
       </c>
       <c r="AF215" t="s" s="2">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="AG215" t="s" s="2">
         <v>79</v>
@@ -28430,10 +28422,10 @@
     </row>
     <row r="216" hidden="true">
       <c r="A216" t="s" s="2">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B216" t="s" s="2">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="C216" s="2"/>
       <c r="D216" t="s" s="2">
@@ -28459,10 +28451,10 @@
         <v>230</v>
       </c>
       <c r="L216" t="s" s="2">
+        <v>747</v>
+      </c>
+      <c r="M216" t="s" s="2">
         <v>748</v>
-      </c>
-      <c r="M216" t="s" s="2">
-        <v>749</v>
       </c>
       <c r="N216" s="2"/>
       <c r="O216" s="2"/>
@@ -28513,7 +28505,7 @@
         <v>78</v>
       </c>
       <c r="AF216" t="s" s="2">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="AG216" t="s" s="2">
         <v>79</v>
@@ -28534,7 +28526,7 @@
         <v>198</v>
       </c>
       <c r="AM216" t="s" s="2">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="AN216" t="s" s="2">
         <v>358</v>
@@ -28545,13 +28537,13 @@
     </row>
     <row r="217" hidden="true">
       <c r="A217" t="s" s="2">
+        <v>751</v>
+      </c>
+      <c r="B217" t="s" s="2">
+        <v>692</v>
+      </c>
+      <c r="C217" t="s" s="2">
         <v>752</v>
-      </c>
-      <c r="B217" t="s" s="2">
-        <v>693</v>
-      </c>
-      <c r="C217" t="s" s="2">
-        <v>753</v>
       </c>
       <c r="D217" t="s" s="2">
         <v>78</v>
@@ -28573,19 +28565,19 @@
         <v>78</v>
       </c>
       <c r="K217" t="s" s="2">
+        <v>753</v>
+      </c>
+      <c r="L217" t="s" s="2">
         <v>754</v>
       </c>
-      <c r="L217" t="s" s="2">
-        <v>755</v>
-      </c>
       <c r="M217" t="s" s="2">
+        <v>695</v>
+      </c>
+      <c r="N217" t="s" s="2">
         <v>696</v>
       </c>
-      <c r="N217" t="s" s="2">
+      <c r="O217" t="s" s="2">
         <v>697</v>
-      </c>
-      <c r="O217" t="s" s="2">
-        <v>698</v>
       </c>
       <c r="P217" t="s" s="2">
         <v>78</v>
@@ -28634,7 +28626,7 @@
         <v>78</v>
       </c>
       <c r="AF217" t="s" s="2">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="AG217" t="s" s="2">
         <v>79</v>
@@ -28646,19 +28638,19 @@
         <v>207</v>
       </c>
       <c r="AJ217" t="s" s="2">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="AK217" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL217" t="s" s="2">
+        <v>701</v>
+      </c>
+      <c r="AM217" t="s" s="2">
         <v>702</v>
       </c>
-      <c r="AM217" t="s" s="2">
+      <c r="AN217" t="s" s="2">
         <v>703</v>
-      </c>
-      <c r="AN217" t="s" s="2">
-        <v>704</v>
       </c>
       <c r="AO217" t="s" s="2">
         <v>78</v>
@@ -28666,10 +28658,10 @@
     </row>
     <row r="218" hidden="true">
       <c r="A218" t="s" s="2">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B218" t="s" s="2">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="C218" s="2"/>
       <c r="D218" t="s" s="2">
@@ -28781,10 +28773,10 @@
     </row>
     <row r="219" hidden="true">
       <c r="A219" t="s" s="2">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B219" t="s" s="2">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C219" s="2"/>
       <c r="D219" t="s" s="2">
@@ -28898,13 +28890,13 @@
     </row>
     <row r="220" hidden="true">
       <c r="A220" t="s" s="2">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="B220" t="s" s="2">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C220" t="s" s="2">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="D220" t="s" s="2">
         <v>78</v>
@@ -28926,13 +28918,13 @@
         <v>78</v>
       </c>
       <c r="K220" t="s" s="2">
+        <v>708</v>
+      </c>
+      <c r="L220" t="s" s="2">
         <v>709</v>
       </c>
-      <c r="L220" t="s" s="2">
+      <c r="M220" t="s" s="2">
         <v>710</v>
-      </c>
-      <c r="M220" t="s" s="2">
-        <v>711</v>
       </c>
       <c r="N220" s="2"/>
       <c r="O220" s="2"/>
@@ -29015,10 +29007,10 @@
     </row>
     <row r="221" hidden="true">
       <c r="A221" t="s" s="2">
+        <v>758</v>
+      </c>
+      <c r="B221" t="s" s="2">
         <v>759</v>
-      </c>
-      <c r="B221" t="s" s="2">
-        <v>760</v>
       </c>
       <c r="C221" s="2"/>
       <c r="D221" t="s" s="2">
@@ -29130,10 +29122,10 @@
     </row>
     <row r="222" hidden="true">
       <c r="A222" t="s" s="2">
+        <v>760</v>
+      </c>
+      <c r="B222" t="s" s="2">
         <v>761</v>
-      </c>
-      <c r="B222" t="s" s="2">
-        <v>762</v>
       </c>
       <c r="C222" s="2"/>
       <c r="D222" t="s" s="2">
@@ -29245,10 +29237,10 @@
     </row>
     <row r="223" hidden="true">
       <c r="A223" t="s" s="2">
+        <v>762</v>
+      </c>
+      <c r="B223" t="s" s="2">
         <v>763</v>
-      </c>
-      <c r="B223" t="s" s="2">
-        <v>764</v>
       </c>
       <c r="C223" s="2"/>
       <c r="D223" t="s" s="2">
@@ -29288,7 +29280,7 @@
       </c>
       <c r="Q223" s="2"/>
       <c r="R223" t="s" s="2">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="S223" t="s" s="2">
         <v>78</v>
@@ -29362,10 +29354,10 @@
     </row>
     <row r="224" hidden="true">
       <c r="A224" t="s" s="2">
+        <v>765</v>
+      </c>
+      <c r="B224" t="s" s="2">
         <v>766</v>
-      </c>
-      <c r="B224" t="s" s="2">
-        <v>767</v>
       </c>
       <c r="C224" s="2"/>
       <c r="D224" t="s" s="2">
@@ -29394,7 +29386,7 @@
         <v>231</v>
       </c>
       <c r="M224" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N224" s="2"/>
       <c r="O224" s="2"/>
@@ -29406,7 +29398,7 @@
         <v>78</v>
       </c>
       <c r="S224" t="s" s="2">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="T224" t="s" s="2">
         <v>78</v>
@@ -29425,7 +29417,7 @@
       </c>
       <c r="Y224" s="2"/>
       <c r="Z224" t="s" s="2">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="AA224" t="s" s="2">
         <v>78</v>
@@ -29475,13 +29467,13 @@
     </row>
     <row r="225" hidden="true">
       <c r="A225" t="s" s="2">
+        <v>769</v>
+      </c>
+      <c r="B225" t="s" s="2">
+        <v>705</v>
+      </c>
+      <c r="C225" t="s" s="2">
         <v>770</v>
-      </c>
-      <c r="B225" t="s" s="2">
-        <v>706</v>
-      </c>
-      <c r="C225" t="s" s="2">
-        <v>771</v>
       </c>
       <c r="D225" t="s" s="2">
         <v>78</v>
@@ -29503,13 +29495,13 @@
         <v>78</v>
       </c>
       <c r="K225" t="s" s="2">
+        <v>771</v>
+      </c>
+      <c r="L225" t="s" s="2">
         <v>772</v>
       </c>
-      <c r="L225" t="s" s="2">
+      <c r="M225" t="s" s="2">
         <v>773</v>
-      </c>
-      <c r="M225" t="s" s="2">
-        <v>774</v>
       </c>
       <c r="N225" s="2"/>
       <c r="O225" s="2"/>
@@ -29592,10 +29584,10 @@
     </row>
     <row r="226" hidden="true">
       <c r="A226" t="s" s="2">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="B226" t="s" s="2">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C226" s="2"/>
       <c r="D226" t="s" s="2">
@@ -29707,10 +29699,10 @@
     </row>
     <row r="227" hidden="true">
       <c r="A227" t="s" s="2">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B227" t="s" s="2">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="C227" s="2"/>
       <c r="D227" t="s" s="2">
@@ -29824,13 +29816,13 @@
     </row>
     <row r="228" hidden="true">
       <c r="A228" t="s" s="2">
+        <v>776</v>
+      </c>
+      <c r="B228" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="C228" t="s" s="2">
         <v>777</v>
-      </c>
-      <c r="B228" t="s" s="2">
-        <v>762</v>
-      </c>
-      <c r="C228" t="s" s="2">
-        <v>778</v>
       </c>
       <c r="D228" t="s" s="2">
         <v>78</v>
@@ -29855,7 +29847,7 @@
         <v>110</v>
       </c>
       <c r="L228" t="s" s="2">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="M228" t="s" s="2">
         <v>201</v>
@@ -29941,10 +29933,10 @@
     </row>
     <row r="229" hidden="true">
       <c r="A229" t="s" s="2">
+        <v>779</v>
+      </c>
+      <c r="B229" t="s" s="2">
         <v>780</v>
-      </c>
-      <c r="B229" t="s" s="2">
-        <v>781</v>
       </c>
       <c r="C229" s="2"/>
       <c r="D229" t="s" s="2">
@@ -30056,10 +30048,10 @@
     </row>
     <row r="230" hidden="true">
       <c r="A230" t="s" s="2">
+        <v>781</v>
+      </c>
+      <c r="B230" t="s" s="2">
         <v>782</v>
-      </c>
-      <c r="B230" t="s" s="2">
-        <v>783</v>
       </c>
       <c r="C230" s="2"/>
       <c r="D230" t="s" s="2">
@@ -30171,10 +30163,10 @@
     </row>
     <row r="231" hidden="true">
       <c r="A231" t="s" s="2">
+        <v>783</v>
+      </c>
+      <c r="B231" t="s" s="2">
         <v>784</v>
-      </c>
-      <c r="B231" t="s" s="2">
-        <v>785</v>
       </c>
       <c r="C231" s="2"/>
       <c r="D231" t="s" s="2">
@@ -30214,7 +30206,7 @@
       </c>
       <c r="Q231" s="2"/>
       <c r="R231" t="s" s="2">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="S231" t="s" s="2">
         <v>78</v>
@@ -30288,10 +30280,10 @@
     </row>
     <row r="232" hidden="true">
       <c r="A232" t="s" s="2">
+        <v>785</v>
+      </c>
+      <c r="B232" t="s" s="2">
         <v>786</v>
-      </c>
-      <c r="B232" t="s" s="2">
-        <v>787</v>
       </c>
       <c r="C232" s="2"/>
       <c r="D232" t="s" s="2">
@@ -30320,7 +30312,7 @@
         <v>231</v>
       </c>
       <c r="M232" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N232" s="2"/>
       <c r="O232" s="2"/>
@@ -30351,7 +30343,7 @@
       </c>
       <c r="Y232" s="2"/>
       <c r="Z232" t="s" s="2">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="AA232" t="s" s="2">
         <v>78</v>
@@ -30401,10 +30393,10 @@
     </row>
     <row r="233" hidden="true">
       <c r="A233" t="s" s="2">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B233" t="s" s="2">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="C233" t="s" s="2">
         <v>209</v>
@@ -30432,7 +30424,7 @@
         <v>110</v>
       </c>
       <c r="L233" t="s" s="2">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="M233" t="s" s="2">
         <v>201</v>
@@ -30518,10 +30510,10 @@
     </row>
     <row r="234" hidden="true">
       <c r="A234" t="s" s="2">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B234" t="s" s="2">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C234" s="2"/>
       <c r="D234" t="s" s="2">
@@ -30633,10 +30625,10 @@
     </row>
     <row r="235" hidden="true">
       <c r="A235" t="s" s="2">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B235" t="s" s="2">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C235" s="2"/>
       <c r="D235" t="s" s="2">
@@ -30748,10 +30740,10 @@
     </row>
     <row r="236" hidden="true">
       <c r="A236" t="s" s="2">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B236" t="s" s="2">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C236" s="2"/>
       <c r="D236" t="s" s="2">
@@ -30865,10 +30857,10 @@
     </row>
     <row r="237" hidden="true">
       <c r="A237" t="s" s="2">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B237" t="s" s="2">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C237" s="2"/>
       <c r="D237" t="s" s="2">
@@ -30897,7 +30889,7 @@
         <v>231</v>
       </c>
       <c r="M237" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N237" s="2"/>
       <c r="O237" s="2"/>
@@ -30980,13 +30972,13 @@
     </row>
     <row r="238" hidden="true">
       <c r="A238" t="s" s="2">
+        <v>794</v>
+      </c>
+      <c r="B238" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="C238" t="s" s="2">
         <v>795</v>
-      </c>
-      <c r="B238" t="s" s="2">
-        <v>762</v>
-      </c>
-      <c r="C238" t="s" s="2">
-        <v>796</v>
       </c>
       <c r="D238" t="s" s="2">
         <v>78</v>
@@ -31097,10 +31089,10 @@
     </row>
     <row r="239" hidden="true">
       <c r="A239" t="s" s="2">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="B239" t="s" s="2">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C239" s="2"/>
       <c r="D239" t="s" s="2">
@@ -31212,10 +31204,10 @@
     </row>
     <row r="240" hidden="true">
       <c r="A240" t="s" s="2">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B240" t="s" s="2">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C240" s="2"/>
       <c r="D240" t="s" s="2">
@@ -31327,10 +31319,10 @@
     </row>
     <row r="241" hidden="true">
       <c r="A241" t="s" s="2">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B241" t="s" s="2">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C241" s="2"/>
       <c r="D241" t="s" s="2">
@@ -31370,7 +31362,7 @@
       </c>
       <c r="Q241" s="2"/>
       <c r="R241" t="s" s="2">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="S241" t="s" s="2">
         <v>78</v>
@@ -31444,10 +31436,10 @@
     </row>
     <row r="242" hidden="true">
       <c r="A242" t="s" s="2">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="B242" t="s" s="2">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C242" s="2"/>
       <c r="D242" t="s" s="2">
@@ -31476,7 +31468,7 @@
         <v>231</v>
       </c>
       <c r="M242" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N242" s="2"/>
       <c r="O242" s="2"/>
@@ -31559,13 +31551,13 @@
     </row>
     <row r="243" hidden="true">
       <c r="A243" t="s" s="2">
+        <v>800</v>
+      </c>
+      <c r="B243" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="C243" t="s" s="2">
         <v>801</v>
-      </c>
-      <c r="B243" t="s" s="2">
-        <v>762</v>
-      </c>
-      <c r="C243" t="s" s="2">
-        <v>802</v>
       </c>
       <c r="D243" t="s" s="2">
         <v>78</v>
@@ -31590,7 +31582,7 @@
         <v>110</v>
       </c>
       <c r="L243" t="s" s="2">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="M243" t="s" s="2">
         <v>201</v>
@@ -31676,10 +31668,10 @@
     </row>
     <row r="244" hidden="true">
       <c r="A244" t="s" s="2">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="B244" t="s" s="2">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C244" s="2"/>
       <c r="D244" t="s" s="2">
@@ -31791,10 +31783,10 @@
     </row>
     <row r="245" hidden="true">
       <c r="A245" t="s" s="2">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B245" t="s" s="2">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C245" s="2"/>
       <c r="D245" t="s" s="2">
@@ -31906,10 +31898,10 @@
     </row>
     <row r="246" hidden="true">
       <c r="A246" t="s" s="2">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B246" t="s" s="2">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C246" s="2"/>
       <c r="D246" t="s" s="2">
@@ -31949,7 +31941,7 @@
       </c>
       <c r="Q246" s="2"/>
       <c r="R246" t="s" s="2">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="S246" t="s" s="2">
         <v>78</v>
@@ -32023,10 +32015,10 @@
     </row>
     <row r="247" hidden="true">
       <c r="A247" t="s" s="2">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B247" t="s" s="2">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C247" s="2"/>
       <c r="D247" t="s" s="2">
@@ -32055,7 +32047,7 @@
         <v>231</v>
       </c>
       <c r="M247" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N247" s="2"/>
       <c r="O247" s="2"/>
@@ -32138,13 +32130,13 @@
     </row>
     <row r="248" hidden="true">
       <c r="A248" t="s" s="2">
+        <v>807</v>
+      </c>
+      <c r="B248" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="C248" t="s" s="2">
         <v>808</v>
-      </c>
-      <c r="B248" t="s" s="2">
-        <v>762</v>
-      </c>
-      <c r="C248" t="s" s="2">
-        <v>809</v>
       </c>
       <c r="D248" t="s" s="2">
         <v>78</v>
@@ -32255,10 +32247,10 @@
     </row>
     <row r="249" hidden="true">
       <c r="A249" t="s" s="2">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="B249" t="s" s="2">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C249" s="2"/>
       <c r="D249" t="s" s="2">
@@ -32370,10 +32362,10 @@
     </row>
     <row r="250" hidden="true">
       <c r="A250" t="s" s="2">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B250" t="s" s="2">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C250" s="2"/>
       <c r="D250" t="s" s="2">
@@ -32485,10 +32477,10 @@
     </row>
     <row r="251" hidden="true">
       <c r="A251" t="s" s="2">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B251" t="s" s="2">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C251" s="2"/>
       <c r="D251" t="s" s="2">
@@ -32528,7 +32520,7 @@
       </c>
       <c r="Q251" s="2"/>
       <c r="R251" t="s" s="2">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="S251" t="s" s="2">
         <v>78</v>
@@ -32602,10 +32594,10 @@
     </row>
     <row r="252" hidden="true">
       <c r="A252" t="s" s="2">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B252" t="s" s="2">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C252" s="2"/>
       <c r="D252" t="s" s="2">
@@ -32634,7 +32626,7 @@
         <v>231</v>
       </c>
       <c r="M252" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N252" s="2"/>
       <c r="O252" s="2"/>
@@ -32717,13 +32709,13 @@
     </row>
     <row r="253" hidden="true">
       <c r="A253" t="s" s="2">
+        <v>813</v>
+      </c>
+      <c r="B253" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="C253" t="s" s="2">
         <v>814</v>
-      </c>
-      <c r="B253" t="s" s="2">
-        <v>762</v>
-      </c>
-      <c r="C253" t="s" s="2">
-        <v>815</v>
       </c>
       <c r="D253" t="s" s="2">
         <v>78</v>
@@ -32748,7 +32740,7 @@
         <v>110</v>
       </c>
       <c r="L253" t="s" s="2">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="M253" t="s" s="2">
         <v>201</v>
@@ -32834,10 +32826,10 @@
     </row>
     <row r="254" hidden="true">
       <c r="A254" t="s" s="2">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B254" t="s" s="2">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C254" s="2"/>
       <c r="D254" t="s" s="2">
@@ -32949,10 +32941,10 @@
     </row>
     <row r="255" hidden="true">
       <c r="A255" t="s" s="2">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="B255" t="s" s="2">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C255" s="2"/>
       <c r="D255" t="s" s="2">
@@ -33064,10 +33056,10 @@
     </row>
     <row r="256" hidden="true">
       <c r="A256" t="s" s="2">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B256" t="s" s="2">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C256" s="2"/>
       <c r="D256" t="s" s="2">
@@ -33107,7 +33099,7 @@
       </c>
       <c r="Q256" s="2"/>
       <c r="R256" t="s" s="2">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="S256" t="s" s="2">
         <v>78</v>
@@ -33181,10 +33173,10 @@
     </row>
     <row r="257" hidden="true">
       <c r="A257" t="s" s="2">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B257" t="s" s="2">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C257" s="2"/>
       <c r="D257" t="s" s="2">
@@ -33213,7 +33205,7 @@
         <v>231</v>
       </c>
       <c r="M257" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N257" s="2"/>
       <c r="O257" s="2"/>
@@ -33296,13 +33288,13 @@
     </row>
     <row r="258" hidden="true">
       <c r="A258" t="s" s="2">
+        <v>820</v>
+      </c>
+      <c r="B258" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="C258" t="s" s="2">
         <v>821</v>
-      </c>
-      <c r="B258" t="s" s="2">
-        <v>762</v>
-      </c>
-      <c r="C258" t="s" s="2">
-        <v>822</v>
       </c>
       <c r="D258" t="s" s="2">
         <v>78</v>
@@ -33327,7 +33319,7 @@
         <v>110</v>
       </c>
       <c r="L258" t="s" s="2">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="M258" t="s" s="2">
         <v>201</v>
@@ -33413,10 +33405,10 @@
     </row>
     <row r="259" hidden="true">
       <c r="A259" t="s" s="2">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="B259" t="s" s="2">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C259" s="2"/>
       <c r="D259" t="s" s="2">
@@ -33528,10 +33520,10 @@
     </row>
     <row r="260" hidden="true">
       <c r="A260" t="s" s="2">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B260" t="s" s="2">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C260" s="2"/>
       <c r="D260" t="s" s="2">
@@ -33643,10 +33635,10 @@
     </row>
     <row r="261" hidden="true">
       <c r="A261" t="s" s="2">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="B261" t="s" s="2">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="C261" s="2"/>
       <c r="D261" t="s" s="2">
@@ -33686,7 +33678,7 @@
       </c>
       <c r="Q261" s="2"/>
       <c r="R261" t="s" s="2">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="S261" t="s" s="2">
         <v>78</v>
@@ -33760,10 +33752,10 @@
     </row>
     <row r="262" hidden="true">
       <c r="A262" t="s" s="2">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="B262" t="s" s="2">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C262" s="2"/>
       <c r="D262" t="s" s="2">
@@ -33792,7 +33784,7 @@
         <v>231</v>
       </c>
       <c r="M262" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N262" s="2"/>
       <c r="O262" s="2"/>
@@ -33875,10 +33867,10 @@
     </row>
     <row r="263" hidden="true">
       <c r="A263" t="s" s="2">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="B263" t="s" s="2">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="C263" s="2"/>
       <c r="D263" t="s" s="2">
@@ -33918,7 +33910,7 @@
       </c>
       <c r="Q263" s="2"/>
       <c r="R263" t="s" s="2">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="S263" t="s" s="2">
         <v>78</v>
@@ -33992,10 +33984,10 @@
     </row>
     <row r="264" hidden="true">
       <c r="A264" t="s" s="2">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="B264" t="s" s="2">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="C264" s="2"/>
       <c r="D264" t="s" s="2">
@@ -34018,13 +34010,13 @@
         <v>78</v>
       </c>
       <c r="K264" t="s" s="2">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="L264" t="s" s="2">
         <v>231</v>
       </c>
       <c r="M264" t="s" s="2">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N264" s="2"/>
       <c r="O264" s="2"/>
@@ -34107,10 +34099,10 @@
     </row>
     <row r="265" hidden="true">
       <c r="A265" t="s" s="2">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="B265" t="s" s="2">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C265" s="2"/>
       <c r="D265" t="s" s="2">
@@ -34136,10 +34128,10 @@
         <v>175</v>
       </c>
       <c r="L265" t="s" s="2">
+        <v>712</v>
+      </c>
+      <c r="M265" t="s" s="2">
         <v>713</v>
-      </c>
-      <c r="M265" t="s" s="2">
-        <v>714</v>
       </c>
       <c r="N265" s="2"/>
       <c r="O265" s="2"/>
@@ -34151,7 +34143,7 @@
         <v>78</v>
       </c>
       <c r="S265" t="s" s="2">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="T265" t="s" s="2">
         <v>78</v>
@@ -34169,37 +34161,37 @@
         <v>316</v>
       </c>
       <c r="Y265" t="s" s="2">
+        <v>714</v>
+      </c>
+      <c r="Z265" t="s" s="2">
         <v>715</v>
       </c>
-      <c r="Z265" t="s" s="2">
+      <c r="AA265" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB265" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC265" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD265" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE265" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF265" t="s" s="2">
         <v>716</v>
       </c>
-      <c r="AA265" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB265" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC265" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD265" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE265" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF265" t="s" s="2">
+      <c r="AG265" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH265" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI265" t="s" s="2">
         <v>717</v>
-      </c>
-      <c r="AG265" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH265" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI265" t="s" s="2">
-        <v>718</v>
       </c>
       <c r="AJ265" t="s" s="2">
         <v>101</v>
@@ -34208,13 +34200,13 @@
         <v>78</v>
       </c>
       <c r="AL265" t="s" s="2">
+        <v>718</v>
+      </c>
+      <c r="AM265" t="s" s="2">
         <v>719</v>
       </c>
-      <c r="AM265" t="s" s="2">
+      <c r="AN265" t="s" s="2">
         <v>720</v>
-      </c>
-      <c r="AN265" t="s" s="2">
-        <v>721</v>
       </c>
       <c r="AO265" t="s" s="2">
         <v>78</v>
@@ -34222,10 +34214,10 @@
     </row>
     <row r="266" hidden="true">
       <c r="A266" t="s" s="2">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B266" t="s" s="2">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C266" s="2"/>
       <c r="D266" t="s" s="2">
@@ -34251,16 +34243,16 @@
         <v>103</v>
       </c>
       <c r="L266" t="s" s="2">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="M266" t="s" s="2">
+        <v>723</v>
+      </c>
+      <c r="N266" t="s" s="2">
         <v>724</v>
       </c>
-      <c r="N266" t="s" s="2">
+      <c r="O266" t="s" s="2">
         <v>725</v>
-      </c>
-      <c r="O266" t="s" s="2">
-        <v>726</v>
       </c>
       <c r="P266" t="s" s="2">
         <v>78</v>
@@ -34309,7 +34301,7 @@
         <v>78</v>
       </c>
       <c r="AF266" t="s" s="2">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="AG266" t="s" s="2">
         <v>79</v>
@@ -34327,10 +34319,10 @@
         <v>78</v>
       </c>
       <c r="AL266" t="s" s="2">
+        <v>727</v>
+      </c>
+      <c r="AM266" t="s" s="2">
         <v>728</v>
-      </c>
-      <c r="AM266" t="s" s="2">
-        <v>729</v>
       </c>
       <c r="AN266" t="s" s="2">
         <v>349</v>
@@ -34341,10 +34333,10 @@
     </row>
     <row r="267" hidden="true">
       <c r="A267" t="s" s="2">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B267" t="s" s="2">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="C267" s="2"/>
       <c r="D267" t="s" s="2">
@@ -34370,16 +34362,16 @@
         <v>175</v>
       </c>
       <c r="L267" t="s" s="2">
+        <v>730</v>
+      </c>
+      <c r="M267" t="s" s="2">
         <v>731</v>
       </c>
-      <c r="M267" t="s" s="2">
-        <v>732</v>
-      </c>
       <c r="N267" t="s" s="2">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="O267" t="s" s="2">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="P267" t="s" s="2">
         <v>78</v>
@@ -34407,28 +34399,28 @@
         <v>316</v>
       </c>
       <c r="Y267" t="s" s="2">
+        <v>734</v>
+      </c>
+      <c r="Z267" t="s" s="2">
         <v>735</v>
       </c>
-      <c r="Z267" t="s" s="2">
+      <c r="AA267" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB267" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC267" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD267" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE267" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF267" t="s" s="2">
         <v>736</v>
-      </c>
-      <c r="AA267" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB267" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC267" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD267" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE267" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF267" t="s" s="2">
-        <v>737</v>
       </c>
       <c r="AG267" t="s" s="2">
         <v>79</v>
@@ -34446,13 +34438,13 @@
         <v>78</v>
       </c>
       <c r="AL267" t="s" s="2">
+        <v>737</v>
+      </c>
+      <c r="AM267" t="s" s="2">
         <v>738</v>
       </c>
-      <c r="AM267" t="s" s="2">
+      <c r="AN267" t="s" s="2">
         <v>739</v>
-      </c>
-      <c r="AN267" t="s" s="2">
-        <v>740</v>
       </c>
       <c r="AO267" t="s" s="2">
         <v>78</v>
@@ -34460,10 +34452,10 @@
     </row>
     <row r="268" hidden="true">
       <c r="A268" t="s" s="2">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B268" t="s" s="2">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="C268" s="2"/>
       <c r="D268" t="s" s="2">
@@ -34486,16 +34478,16 @@
         <v>90</v>
       </c>
       <c r="K268" t="s" s="2">
+        <v>741</v>
+      </c>
+      <c r="L268" t="s" s="2">
         <v>742</v>
       </c>
-      <c r="L268" t="s" s="2">
+      <c r="M268" t="s" s="2">
         <v>743</v>
       </c>
-      <c r="M268" t="s" s="2">
+      <c r="N268" t="s" s="2">
         <v>744</v>
-      </c>
-      <c r="N268" t="s" s="2">
-        <v>745</v>
       </c>
       <c r="O268" s="2"/>
       <c r="P268" t="s" s="2">
@@ -34545,7 +34537,7 @@
         <v>78</v>
       </c>
       <c r="AF268" t="s" s="2">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="AG268" t="s" s="2">
         <v>79</v>
@@ -34577,10 +34569,10 @@
     </row>
     <row r="269" hidden="true">
       <c r="A269" t="s" s="2">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B269" t="s" s="2">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="C269" s="2"/>
       <c r="D269" t="s" s="2">
@@ -34606,10 +34598,10 @@
         <v>230</v>
       </c>
       <c r="L269" t="s" s="2">
+        <v>747</v>
+      </c>
+      <c r="M269" t="s" s="2">
         <v>748</v>
-      </c>
-      <c r="M269" t="s" s="2">
-        <v>749</v>
       </c>
       <c r="N269" s="2"/>
       <c r="O269" s="2"/>
@@ -34660,7 +34652,7 @@
         <v>78</v>
       </c>
       <c r="AF269" t="s" s="2">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="AG269" t="s" s="2">
         <v>79</v>
@@ -34681,7 +34673,7 @@
         <v>198</v>
       </c>
       <c r="AM269" t="s" s="2">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="AN269" t="s" s="2">
         <v>358</v>
@@ -34692,10 +34684,10 @@
     </row>
     <row r="270" hidden="true">
       <c r="A270" t="s" s="2">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B270" t="s" s="2">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="C270" s="2"/>
       <c r="D270" t="s" s="2">
@@ -34718,19 +34710,19 @@
         <v>78</v>
       </c>
       <c r="K270" t="s" s="2">
+        <v>840</v>
+      </c>
+      <c r="L270" t="s" s="2">
         <v>841</v>
       </c>
-      <c r="L270" t="s" s="2">
+      <c r="M270" t="s" s="2">
         <v>842</v>
       </c>
-      <c r="M270" t="s" s="2">
+      <c r="N270" t="s" s="2">
         <v>843</v>
       </c>
-      <c r="N270" t="s" s="2">
+      <c r="O270" t="s" s="2">
         <v>844</v>
-      </c>
-      <c r="O270" t="s" s="2">
-        <v>845</v>
       </c>
       <c r="P270" t="s" s="2">
         <v>78</v>
@@ -34779,7 +34771,7 @@
         <v>78</v>
       </c>
       <c r="AF270" t="s" s="2">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="AG270" t="s" s="2">
         <v>79</v>
@@ -34791,19 +34783,19 @@
         <v>207</v>
       </c>
       <c r="AJ270" t="s" s="2">
+        <v>845</v>
+      </c>
+      <c r="AK270" t="s" s="2">
         <v>846</v>
       </c>
-      <c r="AK270" t="s" s="2">
+      <c r="AL270" t="s" s="2">
         <v>847</v>
       </c>
-      <c r="AL270" t="s" s="2">
+      <c r="AM270" t="s" s="2">
         <v>848</v>
       </c>
-      <c r="AM270" t="s" s="2">
+      <c r="AN270" t="s" s="2">
         <v>849</v>
-      </c>
-      <c r="AN270" t="s" s="2">
-        <v>850</v>
       </c>
       <c r="AO270" t="s" s="2">
         <v>78</v>
@@ -34811,10 +34803,10 @@
     </row>
     <row r="271" hidden="true">
       <c r="A271" t="s" s="2">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B271" t="s" s="2">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="C271" s="2"/>
       <c r="D271" t="s" s="2">
@@ -34837,17 +34829,17 @@
         <v>90</v>
       </c>
       <c r="K271" t="s" s="2">
+        <v>851</v>
+      </c>
+      <c r="L271" t="s" s="2">
         <v>852</v>
       </c>
-      <c r="L271" t="s" s="2">
+      <c r="M271" t="s" s="2">
         <v>853</v>
-      </c>
-      <c r="M271" t="s" s="2">
-        <v>854</v>
       </c>
       <c r="N271" s="2"/>
       <c r="O271" t="s" s="2">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="P271" t="s" s="2">
         <v>78</v>
@@ -34896,7 +34888,7 @@
         <v>78</v>
       </c>
       <c r="AF271" t="s" s="2">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AG271" t="s" s="2">
         <v>79</v>
@@ -34914,10 +34906,10 @@
         <v>78</v>
       </c>
       <c r="AL271" t="s" s="2">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="AM271" t="s" s="2">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="AN271" t="s" s="2">
         <v>107</v>
@@ -34928,10 +34920,10 @@
     </row>
     <row r="272" hidden="true">
       <c r="A272" t="s" s="2">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B272" t="s" s="2">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="C272" s="2"/>
       <c r="D272" t="s" s="2">
@@ -35043,10 +35035,10 @@
     </row>
     <row r="273" hidden="true">
       <c r="A273" t="s" s="2">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B273" t="s" s="2">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="C273" s="2"/>
       <c r="D273" t="s" s="2">
@@ -35160,10 +35152,10 @@
     </row>
     <row r="274" hidden="true">
       <c r="A274" t="s" s="2">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="B274" t="s" s="2">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="C274" s="2"/>
       <c r="D274" t="s" s="2">
@@ -35189,13 +35181,13 @@
         <v>103</v>
       </c>
       <c r="L274" t="s" s="2">
+        <v>859</v>
+      </c>
+      <c r="M274" t="s" s="2">
         <v>860</v>
       </c>
-      <c r="M274" t="s" s="2">
+      <c r="N274" t="s" s="2">
         <v>861</v>
-      </c>
-      <c r="N274" t="s" s="2">
-        <v>862</v>
       </c>
       <c r="O274" s="2"/>
       <c r="P274" t="s" s="2">
@@ -35245,16 +35237,16 @@
         <v>78</v>
       </c>
       <c r="AF274" t="s" s="2">
+        <v>862</v>
+      </c>
+      <c r="AG274" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH274" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AI274" t="s" s="2">
         <v>863</v>
-      </c>
-      <c r="AG274" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH274" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="AI274" t="s" s="2">
-        <v>864</v>
       </c>
       <c r="AJ274" t="s" s="2">
         <v>101</v>
@@ -35277,10 +35269,10 @@
     </row>
     <row r="275" hidden="true">
       <c r="A275" t="s" s="2">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B275" t="s" s="2">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="C275" s="2"/>
       <c r="D275" t="s" s="2">
@@ -35306,13 +35298,13 @@
         <v>136</v>
       </c>
       <c r="L275" t="s" s="2">
+        <v>865</v>
+      </c>
+      <c r="M275" t="s" s="2">
         <v>866</v>
       </c>
-      <c r="M275" t="s" s="2">
+      <c r="N275" t="s" s="2">
         <v>867</v>
-      </c>
-      <c r="N275" t="s" s="2">
-        <v>868</v>
       </c>
       <c r="O275" s="2"/>
       <c r="P275" t="s" s="2">
@@ -35342,7 +35334,7 @@
       </c>
       <c r="Y275" s="2"/>
       <c r="Z275" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="AA275" t="s" s="2">
         <v>78</v>
@@ -35360,7 +35352,7 @@
         <v>78</v>
       </c>
       <c r="AF275" t="s" s="2">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="AG275" t="s" s="2">
         <v>79</v>
@@ -35392,10 +35384,10 @@
     </row>
     <row r="276" hidden="true">
       <c r="A276" t="s" s="2">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B276" t="s" s="2">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="C276" s="2"/>
       <c r="D276" t="s" s="2">
@@ -35421,13 +35413,13 @@
         <v>298</v>
       </c>
       <c r="L276" t="s" s="2">
+        <v>870</v>
+      </c>
+      <c r="M276" t="s" s="2">
         <v>871</v>
       </c>
-      <c r="M276" t="s" s="2">
+      <c r="N276" t="s" s="2">
         <v>872</v>
-      </c>
-      <c r="N276" t="s" s="2">
-        <v>873</v>
       </c>
       <c r="O276" s="2"/>
       <c r="P276" t="s" s="2">
@@ -35477,7 +35469,7 @@
         <v>78</v>
       </c>
       <c r="AF276" t="s" s="2">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="AG276" t="s" s="2">
         <v>79</v>
@@ -35498,7 +35490,7 @@
         <v>78</v>
       </c>
       <c r="AM276" t="s" s="2">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="AN276" t="s" s="2">
         <v>78</v>
@@ -35509,10 +35501,10 @@
     </row>
     <row r="277" hidden="true">
       <c r="A277" t="s" s="2">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B277" t="s" s="2">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="C277" s="2"/>
       <c r="D277" t="s" s="2">
@@ -35538,13 +35530,13 @@
         <v>103</v>
       </c>
       <c r="L277" t="s" s="2">
+        <v>876</v>
+      </c>
+      <c r="M277" t="s" s="2">
         <v>877</v>
       </c>
-      <c r="M277" t="s" s="2">
+      <c r="N277" t="s" s="2">
         <v>878</v>
-      </c>
-      <c r="N277" t="s" s="2">
-        <v>879</v>
       </c>
       <c r="O277" s="2"/>
       <c r="P277" t="s" s="2">
@@ -35594,7 +35586,7 @@
         <v>78</v>
       </c>
       <c r="AF277" t="s" s="2">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="AG277" t="s" s="2">
         <v>79</v>
@@ -35626,10 +35618,10 @@
     </row>
     <row r="278" hidden="true">
       <c r="A278" t="s" s="2">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B278" t="s" s="2">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="C278" s="2"/>
       <c r="D278" t="s" s="2">
@@ -35652,19 +35644,19 @@
         <v>78</v>
       </c>
       <c r="K278" t="s" s="2">
+        <v>881</v>
+      </c>
+      <c r="L278" t="s" s="2">
         <v>882</v>
       </c>
-      <c r="L278" t="s" s="2">
+      <c r="M278" t="s" s="2">
         <v>883</v>
       </c>
-      <c r="M278" t="s" s="2">
+      <c r="N278" t="s" s="2">
         <v>884</v>
       </c>
-      <c r="N278" t="s" s="2">
+      <c r="O278" t="s" s="2">
         <v>885</v>
-      </c>
-      <c r="O278" t="s" s="2">
-        <v>886</v>
       </c>
       <c r="P278" t="s" s="2">
         <v>78</v>
@@ -35713,7 +35705,7 @@
         <v>78</v>
       </c>
       <c r="AF278" t="s" s="2">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="AG278" t="s" s="2">
         <v>79</v>
@@ -35734,7 +35726,7 @@
         <v>78</v>
       </c>
       <c r="AM278" t="s" s="2">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="AN278" t="s" s="2">
         <v>78</v>
@@ -35745,10 +35737,10 @@
     </row>
     <row r="279" hidden="true">
       <c r="A279" t="s" s="2">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B279" t="s" s="2">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C279" s="2"/>
       <c r="D279" t="s" s="2">
@@ -35860,10 +35852,10 @@
     </row>
     <row r="280" hidden="true">
       <c r="A280" t="s" s="2">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B280" t="s" s="2">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="C280" s="2"/>
       <c r="D280" t="s" s="2">
@@ -35977,14 +35969,14 @@
     </row>
     <row r="281" hidden="true">
       <c r="A281" t="s" s="2">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B281" t="s" s="2">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C281" s="2"/>
       <c r="D281" t="s" s="2">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="E281" s="2"/>
       <c r="F281" t="s" s="2">
@@ -36006,10 +35998,10 @@
         <v>110</v>
       </c>
       <c r="L281" t="s" s="2">
+        <v>891</v>
+      </c>
+      <c r="M281" t="s" s="2">
         <v>892</v>
-      </c>
-      <c r="M281" t="s" s="2">
-        <v>893</v>
       </c>
       <c r="N281" t="s" s="2">
         <v>113</v>
@@ -36064,7 +36056,7 @@
         <v>78</v>
       </c>
       <c r="AF281" t="s" s="2">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="AG281" t="s" s="2">
         <v>79</v>
@@ -36096,10 +36088,10 @@
     </row>
     <row r="282" hidden="true">
       <c r="A282" t="s" s="2">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="B282" t="s" s="2">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="C282" s="2"/>
       <c r="D282" t="s" s="2">
@@ -36125,14 +36117,14 @@
         <v>322</v>
       </c>
       <c r="L282" t="s" s="2">
+        <v>895</v>
+      </c>
+      <c r="M282" t="s" s="2">
         <v>896</v>
-      </c>
-      <c r="M282" t="s" s="2">
-        <v>897</v>
       </c>
       <c r="N282" s="2"/>
       <c r="O282" t="s" s="2">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="P282" t="s" s="2">
         <v>78</v>
@@ -36160,11 +36152,11 @@
         <v>157</v>
       </c>
       <c r="Y282" t="s" s="2">
+        <v>898</v>
+      </c>
+      <c r="Z282" t="s" s="2">
         <v>899</v>
       </c>
-      <c r="Z282" t="s" s="2">
-        <v>900</v>
-      </c>
       <c r="AA282" t="s" s="2">
         <v>78</v>
       </c>
@@ -36181,7 +36173,7 @@
         <v>78</v>
       </c>
       <c r="AF282" t="s" s="2">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="AG282" t="s" s="2">
         <v>79</v>
@@ -36202,7 +36194,7 @@
         <v>78</v>
       </c>
       <c r="AM282" t="s" s="2">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="AN282" t="s" s="2">
         <v>78</v>
@@ -36213,10 +36205,10 @@
     </row>
     <row r="283" hidden="true">
       <c r="A283" t="s" s="2">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B283" t="s" s="2">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="C283" s="2"/>
       <c r="D283" t="s" s="2">
@@ -36239,17 +36231,17 @@
         <v>78</v>
       </c>
       <c r="K283" t="s" s="2">
+        <v>902</v>
+      </c>
+      <c r="L283" t="s" s="2">
         <v>903</v>
       </c>
-      <c r="L283" t="s" s="2">
+      <c r="M283" t="s" s="2">
         <v>904</v>
-      </c>
-      <c r="M283" t="s" s="2">
-        <v>905</v>
       </c>
       <c r="N283" s="2"/>
       <c r="O283" t="s" s="2">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="P283" t="s" s="2">
         <v>78</v>
@@ -36298,7 +36290,7 @@
         <v>78</v>
       </c>
       <c r="AF283" t="s" s="2">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="AG283" t="s" s="2">
         <v>79</v>
@@ -36316,10 +36308,10 @@
         <v>78</v>
       </c>
       <c r="AL283" t="s" s="2">
+        <v>906</v>
+      </c>
+      <c r="AM283" t="s" s="2">
         <v>907</v>
-      </c>
-      <c r="AM283" t="s" s="2">
-        <v>908</v>
       </c>
       <c r="AN283" t="s" s="2">
         <v>78</v>
@@ -36330,10 +36322,10 @@
     </row>
     <row r="284" hidden="true">
       <c r="A284" t="s" s="2">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="B284" t="s" s="2">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C284" s="2"/>
       <c r="D284" t="s" s="2">
@@ -36356,17 +36348,17 @@
         <v>78</v>
       </c>
       <c r="K284" t="s" s="2">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="L284" t="s" s="2">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="M284" t="s" s="2">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="N284" s="2"/>
       <c r="O284" t="s" s="2">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="P284" t="s" s="2">
         <v>78</v>
@@ -36415,7 +36407,7 @@
         <v>78</v>
       </c>
       <c r="AF284" t="s" s="2">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="AG284" t="s" s="2">
         <v>79</v>
@@ -36427,19 +36419,19 @@
         <v>207</v>
       </c>
       <c r="AJ284" t="s" s="2">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="AK284" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL284" t="s" s="2">
+        <v>701</v>
+      </c>
+      <c r="AM284" t="s" s="2">
         <v>702</v>
       </c>
-      <c r="AM284" t="s" s="2">
+      <c r="AN284" t="s" s="2">
         <v>703</v>
-      </c>
-      <c r="AN284" t="s" s="2">
-        <v>704</v>
       </c>
       <c r="AO284" t="s" s="2">
         <v>78</v>
@@ -36447,10 +36439,10 @@
     </row>
     <row r="285" hidden="true">
       <c r="A285" t="s" s="2">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="B285" t="s" s="2">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="C285" s="2"/>
       <c r="D285" t="s" s="2">
@@ -36473,19 +36465,19 @@
         <v>78</v>
       </c>
       <c r="K285" t="s" s="2">
+        <v>912</v>
+      </c>
+      <c r="L285" t="s" s="2">
         <v>913</v>
       </c>
-      <c r="L285" t="s" s="2">
+      <c r="M285" t="s" s="2">
+        <v>842</v>
+      </c>
+      <c r="N285" t="s" s="2">
+        <v>843</v>
+      </c>
+      <c r="O285" t="s" s="2">
         <v>914</v>
-      </c>
-      <c r="M285" t="s" s="2">
-        <v>843</v>
-      </c>
-      <c r="N285" t="s" s="2">
-        <v>844</v>
-      </c>
-      <c r="O285" t="s" s="2">
-        <v>915</v>
       </c>
       <c r="P285" t="s" s="2">
         <v>78</v>
@@ -36534,7 +36526,7 @@
         <v>78</v>
       </c>
       <c r="AF285" t="s" s="2">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="AG285" t="s" s="2">
         <v>79</v>
@@ -36552,13 +36544,13 @@
         <v>78</v>
       </c>
       <c r="AL285" t="s" s="2">
+        <v>847</v>
+      </c>
+      <c r="AM285" t="s" s="2">
         <v>848</v>
       </c>
-      <c r="AM285" t="s" s="2">
+      <c r="AN285" t="s" s="2">
         <v>849</v>
-      </c>
-      <c r="AN285" t="s" s="2">
-        <v>850</v>
       </c>
       <c r="AO285" t="s" s="2">
         <v>78</v>
@@ -36566,10 +36558,10 @@
     </row>
     <row r="286" hidden="true">
       <c r="A286" t="s" s="2">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="B286" t="s" s="2">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="C286" s="2"/>
       <c r="D286" t="s" s="2">
@@ -36592,17 +36584,17 @@
         <v>78</v>
       </c>
       <c r="K286" t="s" s="2">
+        <v>916</v>
+      </c>
+      <c r="L286" t="s" s="2">
         <v>917</v>
       </c>
-      <c r="L286" t="s" s="2">
+      <c r="M286" t="s" s="2">
         <v>918</v>
-      </c>
-      <c r="M286" t="s" s="2">
-        <v>919</v>
       </c>
       <c r="N286" s="2"/>
       <c r="O286" t="s" s="2">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="P286" t="s" s="2">
         <v>78</v>
@@ -36651,7 +36643,7 @@
         <v>78</v>
       </c>
       <c r="AF286" t="s" s="2">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="AG286" t="s" s="2">
         <v>79</v>

</xml_diff>

<commit_message>
Mise à jour mss type description (#253) 3cf63edebea4035995c4a399e581e0e803b3cf59
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dp-organization.xlsx
+++ b/main/ig/StructureDefinition-as-dp-organization.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-03T16:26:04+00:00</t>
+    <t>2025-02-11T12:19:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2531,10 +2531,7 @@
   </si>
   <si>
     <t>typeBAL : Type de boîte aux lettres.
-Valeurs possibles :
-ORG pour une BAL organisationnelle;
-APP pour une BAL applicative;
-PER pour une BAL personnelle, rattachée à une personne physique</t>
+Valeurs possibles : ORG | APP | PER | CAB</t>
   </si>
   <si>
     <t>Organization.telecom:mailbox-mss.extension:as-mailbox-mss-metadata.extension:type.id</t>

</xml_diff>